<commit_message>
commit New GreenForm Changes
</commit_message>
<xml_diff>
--- a/OnlinePortal-main/SeleniumTestNgKeywordDriven-main/src/test/resources/testData/LoginData.xlsx
+++ b/OnlinePortal-main/SeleniumTestNgKeywordDriven-main/src/test/resources/testData/LoginData.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\silahi\Downloads\OnlinePortal-main\OnlinePortal-main\SeleniumTestNgKeywordDriven-main\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D64597F-72B4-42AE-B44D-9060FD29E68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B5BA842-9AD4-4121-A993-4B6D09CBAC27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginScenarios" sheetId="1" r:id="rId1"/>
     <sheet name="WellSiteAddress" sheetId="2" r:id="rId2"/>
+    <sheet name="WellSiteAdressold" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="54">
   <si>
     <t>Username</t>
   </si>
@@ -137,13 +138,64 @@
   </si>
   <si>
     <t>4 bagley</t>
+  </si>
+  <si>
+    <t>searchMethod</t>
+  </si>
+  <si>
+    <t>propertyNumber</t>
+  </si>
+  <si>
+    <t>isCorrectionNeeded</t>
+  </si>
+  <si>
+    <t>correctionNotes</t>
+  </si>
+  <si>
+    <t>5 ballymena</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>ownerEmail</t>
+  </si>
+  <si>
+    <t>ownerPhone</t>
+  </si>
+  <si>
+    <t>Test@gmail.com</t>
+  </si>
+  <si>
+    <t>5 BALLYMENA CT CATONSVILLE MD 21228 (Baltimore County)</t>
+  </si>
+  <si>
+    <t>6 BALLYMENA CT BALTIMORE MD 21228-2452 (Baltimore County)</t>
+  </si>
+  <si>
+    <t>6 ballymena</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Need to update the Address</t>
+  </si>
+  <si>
+    <t>isOwnerCorrectionNeeded</t>
+  </si>
+  <si>
+    <t>ownercorrectionNotes</t>
+  </si>
+  <si>
+    <t>test.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,6 +224,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -181,7 +239,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -204,12 +262,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -224,6 +295,28 @@
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -587,23 +680,401 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E4EE9B9-AC72-480E-8959-FB278213B5C4}">
+  <dimension ref="A1:T12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.109375" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="4" max="4" width="62.6640625" customWidth="1"/>
+    <col min="5" max="7" width="49.109375" customWidth="1"/>
+    <col min="8" max="8" width="25.77734375" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
+    <col min="10" max="10" width="21.21875" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" customWidth="1"/>
+    <col min="16" max="16" width="16.33203125" customWidth="1"/>
+    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="18" max="18" width="13.88671875" customWidth="1"/>
+    <col min="19" max="19" width="19.5546875" customWidth="1"/>
+    <col min="20" max="20" width="18.21875" customWidth="1"/>
+    <col min="21" max="21" width="19.21875" customWidth="1"/>
+    <col min="22" max="22" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" t="s">
+        <v>51</v>
+      </c>
+      <c r="H1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" t="s">
+        <v>33</v>
+      </c>
+      <c r="S1" t="s">
+        <v>43</v>
+      </c>
+      <c r="T1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B2" s="6">
+        <v>2001000039</v>
+      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I2">
+        <v>5551234567</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2">
+        <v>1234</v>
+      </c>
+      <c r="M2">
+        <v>123</v>
+      </c>
+      <c r="N2">
+        <v>12</v>
+      </c>
+      <c r="O2">
+        <v>12</v>
+      </c>
+      <c r="P2" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>32</v>
+      </c>
+      <c r="R2" t="s">
+        <v>34</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T2">
+        <v>6402293356</v>
+      </c>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B3" s="6">
+        <v>1901000020</v>
+      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="7"/>
+      <c r="I3">
+        <v>5551234567</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3">
+        <v>1234</v>
+      </c>
+      <c r="M3">
+        <v>123</v>
+      </c>
+      <c r="N3">
+        <v>12</v>
+      </c>
+      <c r="O3">
+        <v>12</v>
+      </c>
+      <c r="P3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R3" t="s">
+        <v>34</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T3">
+        <v>6402293356</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B4" s="6">
+        <v>2101000020</v>
+      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="7"/>
+      <c r="I4">
+        <v>5551234567</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K4" t="s">
+        <v>30</v>
+      </c>
+      <c r="L4">
+        <v>1234</v>
+      </c>
+      <c r="M4">
+        <v>123</v>
+      </c>
+      <c r="N4">
+        <v>12</v>
+      </c>
+      <c r="O4">
+        <v>12</v>
+      </c>
+      <c r="P4" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>32</v>
+      </c>
+      <c r="R4" t="s">
+        <v>34</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T4">
+        <v>6402293356</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B5" s="6">
+        <v>2201000047</v>
+      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="7"/>
+      <c r="I5">
+        <v>5551234567</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" t="s">
+        <v>30</v>
+      </c>
+      <c r="L5">
+        <v>1234</v>
+      </c>
+      <c r="M5">
+        <v>123</v>
+      </c>
+      <c r="N5">
+        <v>12</v>
+      </c>
+      <c r="O5">
+        <v>12</v>
+      </c>
+      <c r="P5" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>32</v>
+      </c>
+      <c r="R5" t="s">
+        <v>34</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T5">
+        <v>6402293356</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B6" s="7"/>
+      <c r="C6" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6">
+        <v>5551234567</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" t="s">
+        <v>30</v>
+      </c>
+      <c r="L6">
+        <v>1234</v>
+      </c>
+      <c r="M6">
+        <v>123</v>
+      </c>
+      <c r="N6">
+        <v>12</v>
+      </c>
+      <c r="O6">
+        <v>12</v>
+      </c>
+      <c r="P6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>32</v>
+      </c>
+      <c r="R6" t="s">
+        <v>34</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="T6">
+        <v>6402293356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B8" s="7"/>
+      <c r="C8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="J6" r:id="rId1" xr:uid="{588519F4-C8EA-4374-9524-12F7069DFDBF}"/>
+    <hyperlink ref="S6" r:id="rId2" xr:uid="{39BD71B8-5577-4A14-88E3-86915BB7EE25}"/>
+    <hyperlink ref="J2" r:id="rId3" xr:uid="{2D2C8D04-1C79-4FCB-BFFC-1B2710EA189A}"/>
+    <hyperlink ref="S2" r:id="rId4" xr:uid="{0D61D504-1F8B-4582-A47F-14ECA5CA452D}"/>
+    <hyperlink ref="J3" r:id="rId5" xr:uid="{8C3A8EF7-81C1-469E-8252-33C52DB75F80}"/>
+    <hyperlink ref="S3" r:id="rId6" xr:uid="{9BCC10D0-EBBD-4A1F-A577-BF0CAC63FE3A}"/>
+    <hyperlink ref="J4" r:id="rId7" xr:uid="{0CF3E60B-A147-4FBE-970E-3D448E4B2648}"/>
+    <hyperlink ref="S4" r:id="rId8" xr:uid="{993DE645-4179-4CC6-8EF1-6947E6229F03}"/>
+    <hyperlink ref="J5" r:id="rId9" xr:uid="{50FBF7CC-385F-4F15-AE49-C27F16F73859}"/>
+    <hyperlink ref="S5" r:id="rId10" xr:uid="{EBF73ACE-AA65-4160-B995-5161252AF37B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId11"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576CF0D3-801C-4239-BB7A-4FC616E273D3}">
   <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.88671875" customWidth="1"/>
-    <col min="2" max="2" width="49.109375" customWidth="1"/>
-    <col min="3" max="3" width="19.21875" customWidth="1"/>
-    <col min="4" max="4" width="32.44140625" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="21.21875" customWidth="1"/>
-    <col min="9" max="9" width="14.33203125" customWidth="1"/>
-    <col min="14" max="14" width="16.33203125" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
-    <col min="16" max="16" width="13.88671875" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -653,7 +1124,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="124.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>36</v>
       </c>
@@ -705,9 +1176,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" xr:uid="{588519F4-C8EA-4374-9524-12F7069DFDBF}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{65B5BDCD-783C-4CA9-B9D8-DAE6AB040E94}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>